<commit_message>
Document Zhou Xiaoyang project coordination and integration contributions
</commit_message>
<xml_diff>
--- a/docs/TradingAgents项目协作表.xlsx
+++ b/docs/TradingAgents项目协作表.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="主时间线" sheetId="1" r:id="R964799645d594114"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新日志" sheetId="2" r:id="R5672a5da267d4dd0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="主时间线" sheetId="1" r:id="R26fe4ac94cce43d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新日志" sheetId="2" r:id="R7e1f196afd744f71"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -119,7 +119,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ProjectUpdates" displayName="ProjectUpdates" ref="A7:M22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ProjectUpdates" displayName="ProjectUpdates" ref="A7:M23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="更新ID"/>
     <x:tableColumn id="2" name="记录日期"/>
@@ -1280,7 +1280,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd10e098176b04afd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb944342dd91241d0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2043,15 +2043,56 @@
         <x:v>原始数据仍走Release；密钥/本地日志/环境不入库；不把计划写成已跑通</x:v>
       </x:c>
     </x:row>
+    <x:row r="23" ht="82.5" customHeight="1">
+      <x:c r="A23" s="11" t="str">
+        <x:v>U016</x:v>
+      </x:c>
+      <x:c r="B23" s="12" t="n">
+        <x:v>46311</x:v>
+      </x:c>
+      <x:c r="C23" s="11" t="str">
+        <x:v>2026-10-16</x:v>
+      </x:c>
+      <x:c r="D23" s="11" t="str">
+        <x:v>D 周晓杨 / 整合 Codex</x:v>
+      </x:c>
+      <x:c r="E23" s="11" t="str">
+        <x:v>T01,T02</x:v>
+      </x:c>
+      <x:c r="F23" s="11" t="str">
+        <x:v>周晓杨确认结构、授权推送side；补充个人贡献与组员归属说明</x:v>
+      </x:c>
+      <x:c r="G23" s="11" t="str">
+        <x:v>完成</x:v>
+      </x:c>
+      <x:c r="H23" s="11" t="str">
+        <x:v>docs/CONTRIBUTIONS.md；README.md；PROGRESS.md</x:v>
+      </x:c>
+      <x:c r="I23" s="11" t="str">
+        <x:v>贡献记录已整理；发布状态以远程回执为准，不把推送授权写成推送成功</x:v>
+      </x:c>
+      <x:c r="J23" s="11" t="str">
+        <x:v>整合 Codex</x:v>
+      </x:c>
+      <x:c r="K23" s="11" t="str">
+        <x:v>将已确认整合提交推送side，并核对远程提交</x:v>
+      </x:c>
+      <x:c r="L23" s="12" t="n">
+        <x:v>46312</x:v>
+      </x:c>
+      <x:c r="M23" s="11" t="str">
+        <x:v>周晓杨贡献涵盖统筹、方案、成果核对、proposal/图整合、协作表；Codex辅助明确披露</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="G8:G22">
+    <x:dataValidation type="list" sqref="G8:G23">
       <x:formula1>"完成,部分完成,失败,受阻"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe677914a6d04595"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc473628165704f9f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>